<commit_message>
Added architecture and code problems to report
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ana\Desktop\Silviu_VVSS\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\!FACULTATE\An 3 Sem 2\vvss\Lab1\MyDrinkShop\docs\Lab01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{79F5A167-7FD6-4747-AFE0-B29E797389FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B3712BF-FFC7-4B8E-8E9A-EB4FB798B1C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="650" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" tabRatio="650" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="7" r:id="rId1"/>
@@ -19,22 +19,11 @@
     <sheet name="Tool-basedCodeAnalysis" sheetId="8" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="71">
   <si>
     <t>Document  Title:</t>
   </si>
@@ -212,12 +201,95 @@
   <si>
     <t>Dumitriu Marian</t>
   </si>
+  <si>
+    <t>A05</t>
+  </si>
+  <si>
+    <t>A02</t>
+  </si>
+  <si>
+    <t>A06</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Clasa de test </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial Unicode MS"/>
+      </rPr>
+      <t>ProductTest</t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <charset val="238"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> este amestecată în arhitectura de producție.</t>
+    </r>
+  </si>
+  <si>
+    <t>Serviciile nu folosesc interfețe, ceea ce creează tight coupling între servicii și controller.</t>
+  </si>
+  <si>
+    <t>A01</t>
+  </si>
+  <si>
+    <t>DrinkShopService încalcă Single Responsibility Principle. Rolul serviciului nu este clar, iar controllerul ar putea folosi subserviciile specifice subsistemelor.</t>
+  </si>
+  <si>
+    <t>Clasa ValidationException nu are nicio linie de asociere sau dependență către vreo altă clasă. Nu este evidențiat dacă clasele Service aruncă erori de tipul ValidationException.</t>
+  </si>
+  <si>
+    <t>ValidationException</t>
+  </si>
+  <si>
+    <t>ProductTest</t>
+  </si>
+  <si>
+    <t>DrinkShopService</t>
+  </si>
+  <si>
+    <t>C12</t>
+  </si>
+  <si>
+    <t>Setterul pentru stocMinim nu se potriveste cu tipul său de date definit la început (ca proprietate).</t>
+  </si>
+  <si>
+    <t>C06</t>
+  </si>
+  <si>
+    <t>Nu există nicio validare că sunt destule elemente parsate în linia respectivă; nu este folosit un block try/catch</t>
+  </si>
+  <si>
+    <t>repository/file/FileProductRepository.java [liniile 21-32]</t>
+  </si>
+  <si>
+    <t>domain/Stoc.java - [linia 43]</t>
+  </si>
+  <si>
+    <t>C07</t>
+  </si>
+  <si>
+    <t>export/CsvExporter.java [liniile 24,25,29]</t>
+  </si>
+  <si>
+    <t>Fișierul csv generat nu este valid. Liniile menționate încalcă structura pe coloane a formatului csv.</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,6 +380,21 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="238"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="5">
@@ -409,7 +496,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -440,6 +527,10 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -482,19 +573,18 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -803,37 +893,37 @@
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J27"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="6"/>
-    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="58.28515625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="58.33203125" style="6" customWidth="1"/>
     <col min="4" max="4" width="17" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.85546875" style="6"/>
+    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" style="6"/>
     <col min="9" max="9" width="21" style="6" customWidth="1"/>
-    <col min="10" max="10" width="14.42578125" style="6" customWidth="1"/>
-    <col min="11" max="16384" width="8.85546875" style="6"/>
+    <col min="10" max="10" width="14.44140625" style="6" customWidth="1"/>
+    <col min="11" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>19</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -842,71 +932,69 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="40" t="s">
+      <c r="I3" s="23" t="s">
         <v>48</v>
       </c>
       <c r="J3" s="17">
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10">
       <c r="C4" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="25" t="s">
+      <c r="D4" s="27" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="25"/>
+      <c r="E4" s="27"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="40" t="s">
+      <c r="I4" s="23" t="s">
         <v>49</v>
       </c>
       <c r="J4" s="3">
         <v>232</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10">
       <c r="C5" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="26" t="s">
+      <c r="D5" s="28" t="s">
         <v>13</v>
       </c>
-      <c r="E5" s="27"/>
+      <c r="E5" s="29"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="40" t="s">
+      <c r="I5" s="23" t="s">
         <v>50</v>
       </c>
       <c r="J5" s="3">
         <v>232</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22" t="s">
-        <v>23</v>
-      </c>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -920,37 +1008,37 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" ht="107.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B10" s="37">
+    <row r="10" spans="1:10" ht="107.25" customHeight="1">
+      <c r="B10" s="22">
         <v>1</v>
       </c>
-      <c r="C10" s="36" t="s">
+      <c r="C10" s="41" t="s">
         <v>33</v>
       </c>
       <c r="D10" s="38" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="39" t="s">
+      <c r="E10" s="38" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="11" spans="1:10" ht="125.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="37">
+    <row r="11" spans="1:10" ht="125.25" customHeight="1">
+      <c r="B11" s="22">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="36" t="s">
+      <c r="C11" s="41" t="s">
         <v>34</v>
       </c>
       <c r="D11" s="38" t="s">
         <v>44</v>
       </c>
-      <c r="E11" s="39" t="s">
+      <c r="E11" s="38" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="1:10" ht="102" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="37">
+    <row r="12" spans="1:10" ht="102" customHeight="1">
+      <c r="B12" s="22">
         <f t="shared" ref="B12:B25" si="0">B11+1</f>
         <v>3</v>
       </c>
@@ -960,12 +1048,12 @@
       <c r="D12" s="38" t="s">
         <v>45</v>
       </c>
-      <c r="E12" s="39" t="s">
+      <c r="E12" s="38" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="13" spans="1:10" ht="169.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="37">
+    <row r="13" spans="1:10" ht="169.5" customHeight="1">
+      <c r="B13" s="22">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
@@ -975,12 +1063,12 @@
       <c r="D13" s="38" t="s">
         <v>46</v>
       </c>
-      <c r="E13" s="39" t="s">
+      <c r="E13" s="38" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="14" spans="1:10" ht="114.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="37">
+    <row r="14" spans="1:10" ht="114.75" customHeight="1">
+      <c r="B14" s="22">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
@@ -990,11 +1078,11 @@
       <c r="D14" s="38" t="s">
         <v>47</v>
       </c>
-      <c r="E14" s="39" t="s">
+      <c r="E14" s="38" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1003,7 +1091,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1012,7 +1100,7 @@
       <c r="D16" s="1"/>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1021,7 +1109,7 @@
       <c r="D17" s="1"/>
       <c r="E17" s="2"/>
     </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1030,7 +1118,7 @@
       <c r="D18" s="3"/>
       <c r="E18" s="15"/>
     </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1039,7 +1127,7 @@
       <c r="D19" s="3"/>
       <c r="E19" s="15"/>
     </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1048,7 +1136,7 @@
       <c r="D20" s="3"/>
       <c r="E20" s="15"/>
     </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1057,7 +1145,7 @@
       <c r="D21" s="3"/>
       <c r="E21" s="15"/>
     </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1066,7 +1154,7 @@
       <c r="D22" s="3"/>
       <c r="E22" s="15"/>
     </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1075,7 +1163,7 @@
       <c r="D23" s="3"/>
       <c r="E23" s="15"/>
     </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1084,7 +1172,7 @@
       <c r="D24" s="3"/>
       <c r="E24" s="15"/>
     </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1093,7 +1181,7 @@
       <c r="D25" s="3"/>
       <c r="E25" s="15"/>
     </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:5">
       <c r="C27" s="11" t="s">
         <v>8</v>
       </c>
@@ -1120,35 +1208,36 @@
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J28"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="6"/>
-    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="4" width="16.28515625" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.85546875" style="6"/>
-    <col min="9" max="9" width="22.140625" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="6"/>
+    <col min="1" max="1" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="19.109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" style="6"/>
+    <col min="9" max="9" width="22.109375" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1157,57 +1246,69 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="17">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="30" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="28"/>
+      <c r="E4" s="30"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I4" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="C5" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D5" s="29" t="s">
+      <c r="D5" s="31" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="30"/>
+      <c r="E5" s="32"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I5" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1221,159 +1322,181 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="58.8" customHeight="1">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="38" t="s">
+        <v>51</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>59</v>
+      </c>
+      <c r="E10" s="39" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="28.8">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="38" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>60</v>
+      </c>
+      <c r="E11" s="40" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="28.8">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B26" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" s="38" t="s">
+        <v>53</v>
+      </c>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="57.6">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="38" t="s">
+        <v>56</v>
+      </c>
+      <c r="D13" s="38" t="s">
+        <v>61</v>
+      </c>
+      <c r="E13" s="38" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+    </row>
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+    </row>
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+    </row>
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+    </row>
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+    </row>
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+    </row>
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+    </row>
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+    </row>
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+    </row>
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+    </row>
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+    </row>
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+    </row>
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+    </row>
+    <row r="28" spans="2:5">
       <c r="C28" s="11" t="s">
         <v>8</v>
       </c>
@@ -1400,36 +1523,36 @@
     <tabColor theme="3" tint="0.59999389629810485"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="6"/>
-    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
-    <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="41.42578125" style="6" customWidth="1"/>
-    <col min="6" max="8" width="8.85546875" style="6"/>
-    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="6"/>
+    <col min="1" max="1" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" style="6" customWidth="1"/>
+    <col min="4" max="4" width="36.109375" style="6" customWidth="1"/>
+    <col min="5" max="5" width="41.44140625" style="6" customWidth="1"/>
+    <col min="6" max="8" width="8.88671875" style="6"/>
+    <col min="9" max="9" width="26.6640625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1438,57 +1561,69 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="17">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="D4" s="31" t="s">
+      <c r="D4" s="33" t="s">
         <v>16</v>
       </c>
-      <c r="E4" s="31"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I4" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="C5" s="16" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="32" t="s">
+      <c r="D5" s="34" t="s">
         <v>11</v>
       </c>
-      <c r="E5" s="33"/>
+      <c r="E5" s="35"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I5" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
-    </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+    </row>
+    <row r="7" spans="1:10">
       <c r="C7" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D7" s="22"/>
-      <c r="E7" s="22"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="D7" s="24"/>
+      <c r="E7" s="24"/>
+    </row>
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1502,195 +1637,213 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" ht="43.2">
       <c r="B10" s="3">
         <v>1</v>
       </c>
-      <c r="C10" s="1"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C10" s="38" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" s="38" t="s">
+        <v>67</v>
+      </c>
+      <c r="E10" s="38" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="43.2">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="2"/>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C11" s="38" t="s">
+        <v>64</v>
+      </c>
+      <c r="D11" s="38" t="s">
+        <v>66</v>
+      </c>
+      <c r="E11" s="38" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="43.2">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C12" s="38" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" s="38" t="s">
+        <v>69</v>
+      </c>
+      <c r="E12" s="38" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="1"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-    </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+    </row>
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="1"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+    </row>
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="1"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-    </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+    </row>
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="1"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+    </row>
+    <row r="17" spans="2:5">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="1"/>
-      <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
-    </row>
-    <row r="18" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+    </row>
+    <row r="18" spans="2:5">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="1"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+    </row>
+    <row r="19" spans="2:5">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="2"/>
-    </row>
-    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+    </row>
+    <row r="20" spans="2:5">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="1"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+    </row>
+    <row r="21" spans="2:5">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="1"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="2"/>
-    </row>
-    <row r="22" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+    </row>
+    <row r="22" spans="2:5">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="1"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-    </row>
-    <row r="23" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+    </row>
+    <row r="23" spans="2:5">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="1"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
-    </row>
-    <row r="24" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+    </row>
+    <row r="24" spans="2:5">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="1"/>
-      <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
-    </row>
-    <row r="25" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+    </row>
+    <row r="25" spans="2:5">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="1"/>
-      <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
-    </row>
-    <row r="26" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+    </row>
+    <row r="26" spans="2:5">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-      <c r="E26" s="2"/>
-    </row>
-    <row r="27" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+    </row>
+    <row r="27" spans="2:5">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="1"/>
-      <c r="D27" s="2"/>
-      <c r="E27" s="1"/>
-    </row>
-    <row r="28" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+    </row>
+    <row r="28" spans="2:5">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="1"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-    </row>
-    <row r="29" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+    </row>
+    <row r="29" spans="2:5">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="1"/>
-      <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
-    </row>
-    <row r="30" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+    </row>
+    <row r="30" spans="2:5">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="1"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-    </row>
-    <row r="32" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+    </row>
+    <row r="32" spans="2:5">
       <c r="C32" s="11" t="s">
         <v>8</v>
       </c>
@@ -1717,37 +1870,37 @@
     <tabColor theme="6" tint="0.79998168889431442"/>
   </sheetPr>
   <dimension ref="A1:J35"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="8.85546875" style="6"/>
-    <col min="2" max="2" width="12.28515625" style="6" customWidth="1"/>
-    <col min="3" max="3" width="16.28515625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="6"/>
+    <col min="2" max="2" width="12.33203125" style="6" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" style="6" customWidth="1"/>
     <col min="4" max="4" width="18" style="6" customWidth="1"/>
-    <col min="5" max="5" width="23.85546875" style="6" customWidth="1"/>
-    <col min="6" max="6" width="16.5703125" style="6" customWidth="1"/>
-    <col min="7" max="8" width="8.85546875" style="6"/>
-    <col min="9" max="9" width="26.7109375" style="6" customWidth="1"/>
-    <col min="10" max="16384" width="8.85546875" style="6"/>
+    <col min="5" max="5" width="23.88671875" style="6" customWidth="1"/>
+    <col min="6" max="6" width="16.5546875" style="6" customWidth="1"/>
+    <col min="7" max="8" width="8.88671875" style="6"/>
+    <col min="9" max="9" width="26.6640625" style="6" customWidth="1"/>
+    <col min="10" max="16384" width="8.88671875" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" ht="15.6">
       <c r="A1" s="4"/>
       <c r="B1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="H1" s="23" t="s">
+      <c r="H1" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="24" t="s">
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="B2" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
+      <c r="C2" s="26"/>
+      <c r="D2" s="26"/>
+      <c r="E2" s="26"/>
       <c r="H2" s="3"/>
       <c r="I2" s="19" t="s">
         <v>30</v>
@@ -1756,47 +1909,59 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10">
       <c r="H3" s="17" t="s">
         <v>20</v>
       </c>
-      <c r="I3" s="17"/>
-      <c r="J3" s="17"/>
-    </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I3" s="23" t="s">
+        <v>48</v>
+      </c>
+      <c r="J3" s="17">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="C4" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D4" s="31"/>
-      <c r="E4" s="31"/>
+      <c r="D4" s="33"/>
+      <c r="E4" s="33"/>
       <c r="H4" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-    </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I4" s="23" t="s">
+        <v>49</v>
+      </c>
+      <c r="J4" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="C5" s="9" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
+      <c r="D5" s="24"/>
+      <c r="E5" s="24"/>
       <c r="H5" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I5" s="3"/>
-      <c r="J5" s="3"/>
-    </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="I5" s="23" t="s">
+        <v>50</v>
+      </c>
+      <c r="J5" s="3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="B6" s="8"/>
       <c r="C6" s="9" t="s">
         <v>1</v>
       </c>
-      <c r="D6" s="22"/>
-      <c r="E6" s="22"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
       <c r="F6" s="20"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10">
       <c r="B9" s="10" t="s">
         <v>4</v>
       </c>
@@ -1813,7 +1978,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10">
       <c r="B10" s="3">
         <v>1</v>
       </c>
@@ -1822,7 +1987,7 @@
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10">
       <c r="B11" s="3">
         <f>B10+1</f>
         <v>2</v>
@@ -1832,7 +1997,7 @@
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10">
       <c r="B12" s="3">
         <f t="shared" ref="B12:B30" si="0">B11+1</f>
         <v>3</v>
@@ -1842,7 +2007,7 @@
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10">
       <c r="B13" s="3">
         <f t="shared" si="0"/>
         <v>4</v>
@@ -1852,7 +2017,7 @@
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10">
       <c r="B14" s="3">
         <f t="shared" si="0"/>
         <v>5</v>
@@ -1862,7 +2027,7 @@
       <c r="E14" s="2"/>
       <c r="F14" s="2"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10">
       <c r="B15" s="3">
         <f t="shared" si="0"/>
         <v>6</v>
@@ -1872,7 +2037,7 @@
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10">
       <c r="B16" s="3">
         <f t="shared" si="0"/>
         <v>7</v>
@@ -1882,7 +2047,7 @@
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
     </row>
-    <row r="17" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="2:6">
       <c r="B17" s="3">
         <f t="shared" si="0"/>
         <v>8</v>
@@ -1892,7 +2057,7 @@
       <c r="E17" s="2"/>
       <c r="F17" s="2"/>
     </row>
-    <row r="18" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="2:6">
       <c r="B18" s="3">
         <f t="shared" si="0"/>
         <v>9</v>
@@ -1902,7 +2067,7 @@
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
     </row>
-    <row r="19" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="2:6">
       <c r="B19" s="3">
         <f t="shared" si="0"/>
         <v>10</v>
@@ -1912,7 +2077,7 @@
       <c r="E19" s="2"/>
       <c r="F19" s="2"/>
     </row>
-    <row r="20" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="2:6">
       <c r="B20" s="3">
         <f t="shared" si="0"/>
         <v>11</v>
@@ -1922,7 +2087,7 @@
       <c r="E20" s="2"/>
       <c r="F20" s="2"/>
     </row>
-    <row r="21" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="2:6">
       <c r="B21" s="3">
         <f t="shared" si="0"/>
         <v>12</v>
@@ -1932,7 +2097,7 @@
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
     </row>
-    <row r="22" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="2:6">
       <c r="B22" s="3">
         <f t="shared" si="0"/>
         <v>13</v>
@@ -1942,7 +2107,7 @@
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
-    <row r="23" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="2:6">
       <c r="B23" s="3">
         <f t="shared" si="0"/>
         <v>14</v>
@@ -1952,7 +2117,7 @@
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
-    <row r="24" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="2:6">
       <c r="B24" s="3">
         <f t="shared" si="0"/>
         <v>15</v>
@@ -1962,7 +2127,7 @@
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
-    <row r="25" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="25" spans="2:6">
       <c r="B25" s="3">
         <f t="shared" si="0"/>
         <v>16</v>
@@ -1972,7 +2137,7 @@
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
-    <row r="26" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="26" spans="2:6">
       <c r="B26" s="3">
         <f t="shared" si="0"/>
         <v>17</v>
@@ -1982,7 +2147,7 @@
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
-    <row r="27" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="27" spans="2:6">
       <c r="B27" s="3">
         <f t="shared" si="0"/>
         <v>18</v>
@@ -1992,7 +2157,7 @@
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
     </row>
-    <row r="28" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="28" spans="2:6">
       <c r="B28" s="3">
         <f t="shared" si="0"/>
         <v>19</v>
@@ -2002,7 +2167,7 @@
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
     </row>
-    <row r="29" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="29" spans="2:6">
       <c r="B29" s="3">
         <f t="shared" si="0"/>
         <v>20</v>
@@ -2012,7 +2177,7 @@
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
     </row>
-    <row r="30" spans="2:6" x14ac:dyDescent="0.25">
+    <row r="30" spans="2:6">
       <c r="B30" s="3">
         <f t="shared" si="0"/>
         <v>21</v>
@@ -2022,15 +2187,15 @@
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
     </row>
-    <row r="32" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="C32" s="34" t="s">
+    <row r="32" spans="2:6">
+      <c r="C32" s="36" t="s">
         <v>32</v>
       </c>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
+      <c r="D32" s="37"/>
+      <c r="E32" s="37"/>
       <c r="F32" s="18"/>
     </row>
-    <row r="35" spans="6:6" x14ac:dyDescent="0.25">
+    <row r="35" spans="6:6">
       <c r="F35" s="21"/>
     </row>
   </sheetData>

</xml_diff>